<commit_message>
UK surveillance: finer <5y bins (36-47/48-59mo), default cap 60mo
User updated UK_prevax xlsx to resolve 36-47 and 48-59mo (was open 36+). 6 bins through <5y:
0.122/0.245/0.416/0.137/0.053/0.027 (steep drop after 2y). Default cap=60 keeps the
high/uniform-care-seeking range while adding the 2-5y drop-off diagnostic (does infection-number
overshoot older-child reinfections?). cap=36/24 still available. design effect ~1.5.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/calibration/UK_prevax_age_2008_2012.xlsx
+++ b/calibration/UK_prevax_age_2008_2012.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aliciakraay/PycharmProjects/ryan_rotasim/rotasim/calibration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C413569-B186-2346-BDDC-6B320CA75C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2C2E3B-B8E7-194E-AC0F-CF4DEAB740E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4060" yWindow="3260" windowWidth="27240" windowHeight="16180" xr2:uid="{79FACC84-1E9A-2E48-85F7-35D1F199E8F3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>&lt;6 m</t>
   </si>
@@ -53,7 +53,10 @@
     <t>24-35 m</t>
   </si>
   <si>
-    <t>36 m +</t>
+    <t>36-47 m</t>
+  </si>
+  <si>
+    <t>48-59 m</t>
   </si>
 </sst>
 </file>
@@ -425,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{478CFB07-2D64-454A-8F14-AF3C06F13353}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -530,19 +533,39 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="C6">
-        <v>158</v>
+        <v>53</v>
       </c>
       <c r="D6">
-        <v>149</v>
+        <v>39</v>
       </c>
       <c r="E6">
-        <v>131</v>
+        <v>26</v>
       </c>
       <c r="F6">
-        <v>94</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
+      <c r="C7">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>15</v>
+      </c>
+      <c r="F7">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>